<commit_message>
fix: mobile map and detail panel layout
</commit_message>
<xml_diff>
--- a/public/data/ISO辞書.xlsx
+++ b/public/data/ISO辞書.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\world_map_project\world-map-news-app\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E11B719-37EA-4710-967F-F44BC21223D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C97F897-7F77-4761-8E75-A4980A85A9F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="204" yWindow="492" windowWidth="20688" windowHeight="8880" xr2:uid="{72963FDC-BDE7-4CC9-B88D-6189461FD1D6}"/>
+    <workbookView xWindow="1380" yWindow="852" windowWidth="21600" windowHeight="11232" xr2:uid="{72963FDC-BDE7-4CC9-B88D-6189461FD1D6}"/>
   </bookViews>
   <sheets>
     <sheet name="ISO辞書" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="749" uniqueCount="746">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="752" uniqueCount="749">
   <si>
     <t>A列</t>
   </si>
@@ -2298,6 +2298,17 @@
     <rPh sb="0" eb="2">
       <t>カンコク</t>
     </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>コソボ</t>
+  </si>
+  <si>
+    <t>Kosovo</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>XKK</t>
     <phoneticPr fontId="2"/>
   </si>
 </sst>
@@ -2697,7 +2708,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{209C7BD9-7B68-4B8D-9F2F-40B67A2A5D16}">
-  <dimension ref="A1:D249"/>
+  <dimension ref="A1:D250"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="16.296875" bestFit="1" customWidth="1"/>
@@ -5449,6 +5460,17 @@
         <v>743</v>
       </c>
     </row>
+    <row r="250" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A250" t="s">
+        <v>746</v>
+      </c>
+      <c r="B250" t="s">
+        <v>748</v>
+      </c>
+      <c r="C250" t="s">
+        <v>747</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>